<commit_message>
Harden institutional framework: Fixed glue code bugs, resolved KeyErrors, added __init__.py files, and restored full scorecard reporting
</commit_message>
<xml_diff>
--- a/reports/institutional_swing_analysis.xlsx
+++ b/reports/institutional_swing_analysis.xlsx
@@ -11,7 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="STRONG_SETUPS" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WATCHLIST" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DOWNTRENDS_AVOID" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="METADATA" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SCORECARD_DETAIL" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="METADATA" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -47,7 +48,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -76,17 +77,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -116,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -133,11 +129,14 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -520,14 +519,14 @@
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="8" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="19" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
     <col width="13" customWidth="1" min="19" max="19"/>
     <col width="8" customWidth="1" min="20" max="20"/>
   </cols>
@@ -641,11 +640,11 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>1246.8</v>
+        <v>1343.4</v>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>3/8</t>
+          <t>2/8</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
@@ -663,9 +662,9 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -673,33 +672,33 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I2" s="6" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>DOJI</t>
+          <t>BEARISH_CANDLE</t>
         </is>
       </c>
       <c r="L2" s="2" t="n">
-        <v>1233.37</v>
+        <v>1308.67</v>
       </c>
       <c r="M2" s="2" t="n">
-        <v>1268.36</v>
+        <v>1362.82</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>1226.62</v>
+        <v>1300.02</v>
       </c>
       <c r="O2" s="2" t="n">
-        <v>1268.36</v>
+        <v>1362.82</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>1.07</v>
+        <v>0.45</v>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
@@ -707,27 +706,27 @@
         </is>
       </c>
       <c r="R2" s="2" t="n">
-        <v>0.938799026455484</v>
+        <v>0.7771419941246168</v>
       </c>
       <c r="S2" s="2" t="n">
-        <v>16470167</v>
+        <v>18507370</v>
       </c>
       <c r="T2" s="2" t="n">
-        <v>22.49</v>
+        <v>28.83</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>BHARTIARTL</t>
         </is>
       </c>
-      <c r="B3" s="7" t="n">
-        <v>1246.8</v>
+      <c r="B3" s="5" t="n">
+        <v>1343.4</v>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>3/8</t>
+          <t>2/8</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -735,7 +734,7 @@
           <t>SKIP / NEUTRAL</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>SIDEWAYS</t>
         </is>
@@ -745,9 +744,9 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -755,47 +754,47 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
-        </is>
-      </c>
-      <c r="J3" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="K3" s="7" t="inlineStr">
-        <is>
-          <t>DOJI</t>
-        </is>
-      </c>
-      <c r="L3" s="7" t="n">
-        <v>1233.37</v>
-      </c>
-      <c r="M3" s="7" t="n">
-        <v>1268.36</v>
-      </c>
-      <c r="N3" s="7" t="n">
-        <v>1226.62</v>
-      </c>
-      <c r="O3" s="7" t="n">
-        <v>1268.36</v>
-      </c>
-      <c r="P3" s="7" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="Q3" s="7" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>BEARISH_CANDLE</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="n">
+        <v>1308.67</v>
+      </c>
+      <c r="M3" s="5" t="n">
+        <v>1362.82</v>
+      </c>
+      <c r="N3" s="5" t="n">
+        <v>1300.02</v>
+      </c>
+      <c r="O3" s="5" t="n">
+        <v>1362.82</v>
+      </c>
+      <c r="P3" s="5" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
         <is>
           <t>POOR</t>
         </is>
       </c>
-      <c r="R3" s="7" t="n">
-        <v>0.938799026455484</v>
-      </c>
-      <c r="S3" s="7" t="n">
-        <v>16470167</v>
-      </c>
-      <c r="T3" s="7" t="n">
-        <v>22.49</v>
+      <c r="R3" s="5" t="n">
+        <v>0.7771419941246168</v>
+      </c>
+      <c r="S3" s="5" t="n">
+        <v>18507370</v>
+      </c>
+      <c r="T3" s="5" t="n">
+        <v>28.83</v>
       </c>
     </row>
     <row r="4">
@@ -805,11 +804,11 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1246.8</v>
+        <v>1343.4</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>3/8</t>
+          <t>2/8</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -827,9 +826,9 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -837,33 +836,33 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="J4" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>DOJI</t>
+          <t>BEARISH_CANDLE</t>
         </is>
       </c>
       <c r="L4" s="2" t="n">
-        <v>1233.37</v>
+        <v>1308.67</v>
       </c>
       <c r="M4" s="2" t="n">
-        <v>1268.36</v>
+        <v>1362.82</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>1226.62</v>
+        <v>1300.02</v>
       </c>
       <c r="O4" s="2" t="n">
-        <v>1268.36</v>
+        <v>1362.82</v>
       </c>
       <c r="P4" s="2" t="n">
-        <v>1.07</v>
+        <v>0.45</v>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
@@ -871,27 +870,27 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>0.938799026455484</v>
+        <v>0.7771419941246168</v>
       </c>
       <c r="S4" s="2" t="n">
-        <v>16470167</v>
+        <v>18507370</v>
       </c>
       <c r="T4" s="2" t="n">
-        <v>22.49</v>
+        <v>28.83</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>LT</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n">
-        <v>1246.8</v>
+      <c r="B5" s="5" t="n">
+        <v>1343.4</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>3/8</t>
+          <t>2/8</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -899,7 +898,7 @@
           <t>SKIP / NEUTRAL</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>SIDEWAYS</t>
         </is>
@@ -909,9 +908,9 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
@@ -919,47 +918,47 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
-        </is>
-      </c>
-      <c r="J5" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="K5" s="7" t="inlineStr">
-        <is>
-          <t>DOJI</t>
-        </is>
-      </c>
-      <c r="L5" s="7" t="n">
-        <v>1233.37</v>
-      </c>
-      <c r="M5" s="7" t="n">
-        <v>1268.36</v>
-      </c>
-      <c r="N5" s="7" t="n">
-        <v>1226.62</v>
-      </c>
-      <c r="O5" s="7" t="n">
-        <v>1268.36</v>
-      </c>
-      <c r="P5" s="7" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="Q5" s="7" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>BEARISH_CANDLE</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>1308.67</v>
+      </c>
+      <c r="M5" s="5" t="n">
+        <v>1362.82</v>
+      </c>
+      <c r="N5" s="5" t="n">
+        <v>1300.02</v>
+      </c>
+      <c r="O5" s="5" t="n">
+        <v>1362.82</v>
+      </c>
+      <c r="P5" s="5" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="Q5" s="5" t="inlineStr">
         <is>
           <t>POOR</t>
         </is>
       </c>
-      <c r="R5" s="7" t="n">
-        <v>0.938799026455484</v>
-      </c>
-      <c r="S5" s="7" t="n">
-        <v>16470167</v>
-      </c>
-      <c r="T5" s="7" t="n">
-        <v>22.49</v>
+      <c r="R5" s="5" t="n">
+        <v>0.7771419941246168</v>
+      </c>
+      <c r="S5" s="5" t="n">
+        <v>18507370</v>
+      </c>
+      <c r="T5" s="5" t="n">
+        <v>28.83</v>
       </c>
     </row>
     <row r="6">
@@ -969,11 +968,11 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1246.8</v>
+        <v>1343.4</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>3/8</t>
+          <t>2/8</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -991,9 +990,9 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>YES</t>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -1001,33 +1000,33 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
         </is>
       </c>
       <c r="J6" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>DOJI</t>
+          <t>BEARISH_CANDLE</t>
         </is>
       </c>
       <c r="L6" s="2" t="n">
-        <v>1233.37</v>
+        <v>1308.67</v>
       </c>
       <c r="M6" s="2" t="n">
-        <v>1268.36</v>
+        <v>1362.82</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>1226.62</v>
+        <v>1300.02</v>
       </c>
       <c r="O6" s="2" t="n">
-        <v>1268.36</v>
+        <v>1362.82</v>
       </c>
       <c r="P6" s="2" t="n">
-        <v>1.07</v>
+        <v>0.45</v>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
@@ -1035,13 +1034,13 @@
         </is>
       </c>
       <c r="R6" s="2" t="n">
-        <v>0.938799026455484</v>
+        <v>0.7771419941246168</v>
       </c>
       <c r="S6" s="2" t="n">
-        <v>16470167</v>
+        <v>18507370</v>
       </c>
       <c r="T6" s="2" t="n">
-        <v>22.49</v>
+        <v>28.83</v>
       </c>
     </row>
   </sheetData>
@@ -1469,6 +1468,1184 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Symbol</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>CMP</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Criterion</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C2" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>Uptrend Confirmed (HH + HL on Daily)</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>Mixed swing points – no clear trend bias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Price at Proven Support Zone</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Nearest support: ₹1308.67</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Bullish Reversal Candle at Support</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH_CANDLE – Solid red candle – sellers in control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Support Zone Reaction Count ≥ 2</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>MET</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Touch count: 7 (Major Zone)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>RR Ratio ≥ 1.5 to First Target</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>RR T1: 0.45 (POOR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Clear Path to T1 (No Major Resistance)</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>T1 resistance: ₹1362.82</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Consolidation / Breakout Structure</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>MET</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Inside bar or low-volatility compression visible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>SBIN</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Volume Expansion on Signal Candle</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Last vol: 3,381,205 vs 20-day avg: 18,507,370</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Uptrend Confirmed (HH + HL on Daily)</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Mixed swing points – no clear trend bias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Price at Proven Support Zone</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Nearest support: ₹1308.67</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Bullish Reversal Candle at Support</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH_CANDLE – Solid red candle – sellers in control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Support Zone Reaction Count ≥ 2</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>MET</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>Touch count: 7 (Major Zone)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>RR Ratio ≥ 1.5 to First Target</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>RR T1: 0.45 (POOR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Clear Path to T1 (No Major Resistance)</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>T1 resistance: ₹1362.82</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Consolidation / Breakout Structure</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>MET</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Inside bar or low-volatility compression visible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Volume Expansion on Signal Candle</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Last vol: 3,381,205 vs 20-day avg: 18,507,370</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C20" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>Uptrend Confirmed (HH + HL on Daily)</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>Mixed swing points – no clear trend bias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Price at Proven Support Zone</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>Nearest support: ₹1308.67</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>Bullish Reversal Candle at Support</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH_CANDLE – Solid red candle – sellers in control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Support Zone Reaction Count ≥ 2</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr">
+        <is>
+          <t>MET</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Touch count: 7 (Major Zone)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>RR Ratio ≥ 1.5 to First Target</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>RR T1: 0.45 (POOR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Clear Path to T1 (No Major Resistance)</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>T1 resistance: ₹1362.82</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C26" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>Consolidation / Breakout Structure</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>MET</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Inside bar or low-volatility compression visible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>ITC</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Volume Expansion on Signal Candle</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Last vol: 3,381,205 vs 20-day avg: 18,507,370</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>Uptrend Confirmed (HH + HL on Daily)</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>Mixed swing points – no clear trend bias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C30" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>Price at Proven Support Zone</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F30" s="6" t="inlineStr">
+        <is>
+          <t>Nearest support: ₹1308.67</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>Bullish Reversal Candle at Support</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH_CANDLE – Solid red candle – sellers in control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Support Zone Reaction Count ≥ 2</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>MET</t>
+        </is>
+      </c>
+      <c r="F32" s="6" t="inlineStr">
+        <is>
+          <t>Touch count: 7 (Major Zone)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C33" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>RR Ratio ≥ 1.5 to First Target</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>RR T1: 0.45 (POOR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C34" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>Clear Path to T1 (No Major Resistance)</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F34" s="6" t="inlineStr">
+        <is>
+          <t>T1 resistance: ₹1362.82</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C35" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>Consolidation / Breakout Structure</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>MET</t>
+        </is>
+      </c>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>Inside bar or low-volatility compression visible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>LT</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C36" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>Volume Expansion on Signal Candle</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F36" s="6" t="inlineStr">
+        <is>
+          <t>Last vol: 3,381,205 vs 20-day avg: 18,507,370</t>
+        </is>
+      </c>
+    </row>
+    <row r="37"/>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C38" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>Uptrend Confirmed (HH + HL on Daily)</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>Mixed swing points – no clear trend bias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C39" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>Price at Proven Support Zone</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>Nearest support: ₹1308.67</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C40" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>Bullish Reversal Candle at Support</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>BEARISH_CANDLE – Solid red candle – sellers in control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C41" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D41" s="6" t="inlineStr">
+        <is>
+          <t>Support Zone Reaction Count ≥ 2</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>MET</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>Touch count: 7 (Major Zone)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C42" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>RR Ratio ≥ 1.5 to First Target</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="inlineStr">
+        <is>
+          <t>RR T1: 0.45 (POOR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C43" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>Clear Path to T1 (No Major Resistance)</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>T1 resistance: ₹1362.82</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C44" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>Consolidation / Breakout Structure</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>MET</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>Inside bar or low-volatility compression visible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="n">
+        <v>1343.4</v>
+      </c>
+      <c r="C45" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D45" s="6" t="inlineStr">
+        <is>
+          <t>Volume Expansion on Signal Candle</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>Last vol: 3,381,205 vs 20-day avg: 18,507,370</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1477,7 +2654,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Institutional Swing Analyzer – Run Metadata</t>
         </is>
@@ -1485,120 +2662,120 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Report Generated</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>15-May-2026 09:20:43</t>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>15-May-2026 09:43:15</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Analysis Framework</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Institutional Swing Analyzer v2.0</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Universe</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>NSE Equities (India)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Timeframe</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Daily (1D)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Lookback Period</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>6 Months</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Stocks Scanned</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Processing Time (s)</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>0.7</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Capital Assumed</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>₹500,000</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>Risk Per Trade</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>1.0%</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>SEBI Disclaimer</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>This report is for educational purposes only. Data may have a 30-day lag for unregistered entities. Not investment advice. Consult a SEBI-registered advisor.</t>
         </is>

</xml_diff>

<commit_message>
Final institutional hardening: Resolved pattern serialization issues, added backtest package init, and normalized report paths
</commit_message>
<xml_diff>
--- a/reports/institutional_swing_analysis.xlsx
+++ b/reports/institutional_swing_analysis.xlsx
@@ -77,12 +77,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -112,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -129,13 +129,16 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -506,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T6"/>
+  <dimension ref="A1:T5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -636,15 +639,15 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>SBIN</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>1343.4</v>
+        <v>1250.4</v>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>2/8</t>
+          <t>3/8</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
@@ -662,149 +665,149 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>INDECISION</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>1233.37</v>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>1268.36</v>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>1226.61</v>
+      </c>
+      <c r="O2" s="2" t="n">
+        <v>1268.36</v>
+      </c>
+      <c r="P2" s="2" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>POOR</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="n">
+        <v>0.9386129148029262</v>
+      </c>
+      <c r="S2" s="2" t="n">
+        <v>16516425</v>
+      </c>
+      <c r="T2" s="2" t="n">
+        <v>22.52</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>1250.4</v>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>3/8</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>SKIP / NEUTRAL</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>SIDEWAYS</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH_CANDLE</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="n">
-        <v>1308.67</v>
-      </c>
-      <c r="M2" s="2" t="n">
-        <v>1362.82</v>
-      </c>
-      <c r="N2" s="2" t="n">
-        <v>1300.02</v>
-      </c>
-      <c r="O2" s="2" t="n">
-        <v>1362.82</v>
-      </c>
-      <c r="P2" s="2" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>INDECISION</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="n">
+        <v>1233.37</v>
+      </c>
+      <c r="M3" s="6" t="n">
+        <v>1268.36</v>
+      </c>
+      <c r="N3" s="6" t="n">
+        <v>1226.61</v>
+      </c>
+      <c r="O3" s="6" t="n">
+        <v>1268.36</v>
+      </c>
+      <c r="P3" s="6" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="Q3" s="6" t="inlineStr">
         <is>
           <t>POOR</t>
         </is>
       </c>
-      <c r="R2" s="2" t="n">
-        <v>0.7771419941246168</v>
-      </c>
-      <c r="S2" s="2" t="n">
-        <v>18507370</v>
-      </c>
-      <c r="T2" s="2" t="n">
-        <v>28.83</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>BHARTIARTL</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>2/8</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>SKIP / NEUTRAL</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>SIDEWAYS</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="J3" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="5" t="inlineStr">
-        <is>
-          <t>BEARISH_CANDLE</t>
-        </is>
-      </c>
-      <c r="L3" s="5" t="n">
-        <v>1308.67</v>
-      </c>
-      <c r="M3" s="5" t="n">
-        <v>1362.82</v>
-      </c>
-      <c r="N3" s="5" t="n">
-        <v>1300.02</v>
-      </c>
-      <c r="O3" s="5" t="n">
-        <v>1362.82</v>
-      </c>
-      <c r="P3" s="5" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="Q3" s="5" t="inlineStr">
-        <is>
-          <t>POOR</t>
-        </is>
-      </c>
-      <c r="R3" s="5" t="n">
-        <v>0.7771419941246168</v>
-      </c>
-      <c r="S3" s="5" t="n">
-        <v>18507370</v>
-      </c>
-      <c r="T3" s="5" t="n">
-        <v>28.83</v>
+      <c r="R3" s="6" t="n">
+        <v>0.9386129148029262</v>
+      </c>
+      <c r="S3" s="6" t="n">
+        <v>16516425</v>
+      </c>
+      <c r="T3" s="6" t="n">
+        <v>22.52</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ITC</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1343.4</v>
+        <v>1343</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
@@ -862,7 +865,7 @@
         <v>1362.82</v>
       </c>
       <c r="P4" s="2" t="n">
-        <v>0.45</v>
+        <v>0.46</v>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
@@ -870,23 +873,23 @@
         </is>
       </c>
       <c r="R4" s="2" t="n">
-        <v>0.7771419941246168</v>
+        <v>0.776996003267866</v>
       </c>
       <c r="S4" s="2" t="n">
-        <v>18507370</v>
+        <v>18517099</v>
       </c>
       <c r="T4" s="2" t="n">
         <v>28.83</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>LT</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n">
-        <v>1343.4</v>
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>1343</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
@@ -898,7 +901,7 @@
           <t>SKIP / NEUTRAL</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>SIDEWAYS</t>
         </is>
@@ -923,123 +926,41 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="J5" s="5" t="n">
+      <c r="J5" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="K5" s="6" t="inlineStr">
         <is>
           <t>BEARISH_CANDLE</t>
         </is>
       </c>
-      <c r="L5" s="5" t="n">
+      <c r="L5" s="6" t="n">
         <v>1308.67</v>
       </c>
-      <c r="M5" s="5" t="n">
+      <c r="M5" s="6" t="n">
         <v>1362.82</v>
       </c>
-      <c r="N5" s="5" t="n">
+      <c r="N5" s="6" t="n">
         <v>1300.02</v>
       </c>
-      <c r="O5" s="5" t="n">
+      <c r="O5" s="6" t="n">
         <v>1362.82</v>
       </c>
-      <c r="P5" s="5" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="Q5" s="5" t="inlineStr">
+      <c r="P5" s="6" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="Q5" s="6" t="inlineStr">
         <is>
           <t>POOR</t>
         </is>
       </c>
-      <c r="R5" s="5" t="n">
-        <v>0.7771419941246168</v>
-      </c>
-      <c r="S5" s="5" t="n">
-        <v>18507370</v>
-      </c>
-      <c r="T5" s="5" t="n">
-        <v>28.83</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>ASIANPAINT</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>2/8</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>SKIP / NEUTRAL</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>SIDEWAYS</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>BEARISH_CANDLE</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="n">
-        <v>1308.67</v>
-      </c>
-      <c r="M6" s="2" t="n">
-        <v>1362.82</v>
-      </c>
-      <c r="N6" s="2" t="n">
-        <v>1300.02</v>
-      </c>
-      <c r="O6" s="2" t="n">
-        <v>1362.82</v>
-      </c>
-      <c r="P6" s="2" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="Q6" s="2" t="inlineStr">
-        <is>
-          <t>POOR</t>
-        </is>
-      </c>
-      <c r="R6" s="2" t="n">
-        <v>0.7771419941246168</v>
-      </c>
-      <c r="S6" s="2" t="n">
-        <v>18507370</v>
-      </c>
-      <c r="T6" s="2" t="n">
+      <c r="R5" s="6" t="n">
+        <v>0.776996003267866</v>
+      </c>
+      <c r="S5" s="6" t="n">
+        <v>18517099</v>
+      </c>
+      <c r="T5" s="6" t="n">
         <v>28.83</v>
       </c>
     </row>
@@ -1468,7 +1389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1512,1126 +1433,901 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>SBIN</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C2" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>1250.4</v>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>Uptrend Confirmed (HH + HL on Daily)</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>NOT MET</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>Mixed swing points – no clear trend bias.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>SBIN</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C3" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>1250.4</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>Price at Proven Support Zone</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>MET</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Nearest support: ₹1233.37</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>1250.4</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Bullish Reversal Candle at Support</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>NOT MET</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>Nearest support: ₹1308.67</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>SBIN</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C4" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Bullish Reversal Candle at Support</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>INDECISION – No strong pattern detected – mixed signals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>1250.4</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Support Zone Reaction Count ≥ 2</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>MET</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Touch count: 10 (Major Zone)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>1250.4</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>RR Ratio ≥ 1.5 to First Target</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>NOT MET</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>BEARISH_CANDLE – Solid red candle – sellers in control.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>SBIN</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>Support Zone Reaction Count ≥ 2</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>RR T1: 0.76 (POOR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>1250.4</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Clear Path to T1 (No Major Resistance)</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>T1 resistance: ₹1268.36</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>1250.4</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Consolidation / Breakout Structure</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>MET</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>Touch count: 7 (Major Zone)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>SBIN</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>RR Ratio ≥ 1.5 to First Target</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Inside bar or low-volatility compression visible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>BHARTIARTL</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>1250.4</v>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Volume Expansion on Signal Candle</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>NOT MET</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>RR T1: 0.45 (POOR)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>SBIN</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Clear Path to T1 (No Major Resistance)</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>NOT MET</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>T1 resistance: ₹1362.82</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>SBIN</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>Consolidation / Breakout Structure</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>MET</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>Inside bar or low-volatility compression visible.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>SBIN</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Volume Expansion on Signal Candle</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>NOT MET</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>Last vol: 3,381,205 vs 20-day avg: 18,507,370</t>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Last vol: 1,828,318 vs 20-day avg: 16,516,425</t>
         </is>
       </c>
     </row>
     <row r="10"/>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>BHARTIARTL</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C11" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>1250.4</v>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>Uptrend Confirmed (HH + HL on Daily)</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>NOT MET</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>Mixed swing points – no clear trend bias.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>BHARTIARTL</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C12" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>1250.4</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>Price at Proven Support Zone</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>MET</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Nearest support: ₹1233.37</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>1250.4</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Bullish Reversal Candle at Support</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>NOT MET</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Nearest support: ₹1308.67</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>BHARTIARTL</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>Bullish Reversal Candle at Support</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>INDECISION – No strong pattern detected – mixed signals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>1250.4</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Support Zone Reaction Count ≥ 2</t>
+        </is>
+      </c>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>MET</t>
+        </is>
+      </c>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>Touch count: 10 (Major Zone)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>1250.4</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>RR Ratio ≥ 1.5 to First Target</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>NOT MET</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>BEARISH_CANDLE – Solid red candle – sellers in control.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>BHARTIARTL</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C14" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>Support Zone Reaction Count ≥ 2</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
+      <c r="F15" s="7" t="inlineStr">
+        <is>
+          <t>RR T1: 0.76 (POOR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>1250.4</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>Clear Path to T1 (No Major Resistance)</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>NOT MET</t>
+        </is>
+      </c>
+      <c r="F16" s="7" t="inlineStr">
+        <is>
+          <t>T1 resistance: ₹1268.36</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>1250.4</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Consolidation / Breakout Structure</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
         <is>
           <t>MET</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>Touch count: 7 (Major Zone)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>BHARTIARTL</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C15" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>RR Ratio ≥ 1.5 to First Target</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Inside bar or low-volatility compression visible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>ASIANPAINT</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="n">
+        <v>1250.4</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>Volume Expansion on Signal Candle</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>NOT MET</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>RR T1: 0.45 (POOR)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>BHARTIARTL</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C16" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>Clear Path to T1 (No Major Resistance)</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>NOT MET</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>T1 resistance: ₹1362.82</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>BHARTIARTL</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C17" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>Consolidation / Breakout Structure</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>MET</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>Inside bar or low-volatility compression visible.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>BHARTIARTL</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C18" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>Volume Expansion on Signal Candle</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>NOT MET</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>Last vol: 3,381,205 vs 20-day avg: 18,507,370</t>
+      <c r="F18" s="7" t="inlineStr">
+        <is>
+          <t>Last vol: 1,828,318 vs 20-day avg: 16,516,425</t>
         </is>
       </c>
     </row>
     <row r="19"/>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>ITC</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C20" s="6" t="n">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>1343</v>
+      </c>
+      <c r="C20" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>Uptrend Confirmed (HH + HL on Daily)</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="E20" s="8" t="inlineStr">
         <is>
           <t>NOT MET</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>Mixed swing points – no clear trend bias.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>ITC</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C21" s="6" t="n">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>1343</v>
+      </c>
+      <c r="C21" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D21" s="6" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>Price at Proven Support Zone</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>NOT MET</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="F21" s="7" t="inlineStr">
         <is>
           <t>Nearest support: ₹1308.67</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>ITC</t>
-        </is>
-      </c>
-      <c r="B22" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C22" s="6" t="n">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>1343</v>
+      </c>
+      <c r="C22" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D22" s="6" t="inlineStr">
+      <c r="D22" s="7" t="inlineStr">
         <is>
           <t>Bullish Reversal Candle at Support</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="E22" s="8" t="inlineStr">
         <is>
           <t>NOT MET</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F22" s="7" t="inlineStr">
         <is>
           <t>BEARISH_CANDLE – Solid red candle – sellers in control.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>ITC</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C23" s="6" t="n">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n">
+        <v>1343</v>
+      </c>
+      <c r="C23" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D23" s="6" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>Support Zone Reaction Count ≥ 2</t>
         </is>
       </c>
-      <c r="E23" s="8" t="inlineStr">
+      <c r="E23" s="9" t="inlineStr">
         <is>
           <t>MET</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="F23" s="7" t="inlineStr">
         <is>
           <t>Touch count: 7 (Major Zone)</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>ITC</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C24" s="6" t="n">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="n">
+        <v>1343</v>
+      </c>
+      <c r="C24" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D24" s="6" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t>RR Ratio ≥ 1.5 to First Target</t>
         </is>
       </c>
-      <c r="E24" s="7" t="inlineStr">
+      <c r="E24" s="8" t="inlineStr">
         <is>
           <t>NOT MET</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>RR T1: 0.45 (POOR)</t>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>RR T1: 0.46 (POOR)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>ITC</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C25" s="6" t="n">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>1343</v>
+      </c>
+      <c r="C25" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D25" s="6" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>Clear Path to T1 (No Major Resistance)</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr">
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>NOT MET</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="F25" s="7" t="inlineStr">
         <is>
           <t>T1 resistance: ₹1362.82</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>ITC</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C26" s="6" t="n">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>1343</v>
+      </c>
+      <c r="C26" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D26" s="6" t="inlineStr">
+      <c r="D26" s="7" t="inlineStr">
         <is>
           <t>Consolidation / Breakout Structure</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="E26" s="9" t="inlineStr">
         <is>
           <t>MET</t>
         </is>
       </c>
-      <c r="F26" s="6" t="inlineStr">
+      <c r="F26" s="7" t="inlineStr">
         <is>
           <t>Inside bar or low-volatility compression visible.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>ITC</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C27" s="6" t="n">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>HDFCBANK</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>1343</v>
+      </c>
+      <c r="C27" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D27" s="6" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>Volume Expansion on Signal Candle</t>
         </is>
       </c>
-      <c r="E27" s="7" t="inlineStr">
+      <c r="E27" s="8" t="inlineStr">
         <is>
           <t>NOT MET</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
-        <is>
-          <t>Last vol: 3,381,205 vs 20-day avg: 18,507,370</t>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>Last vol: 3,575,784 vs 20-day avg: 18,517,099</t>
         </is>
       </c>
     </row>
     <row r="28"/>
     <row r="29">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>LT</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C29" s="6" t="n">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="n">
+        <v>1343</v>
+      </c>
+      <c r="C29" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D29" s="6" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>Uptrend Confirmed (HH + HL on Daily)</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr">
+      <c r="E29" s="8" t="inlineStr">
         <is>
           <t>NOT MET</t>
         </is>
       </c>
-      <c r="F29" s="6" t="inlineStr">
+      <c r="F29" s="7" t="inlineStr">
         <is>
           <t>Mixed swing points – no clear trend bias.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>LT</t>
-        </is>
-      </c>
-      <c r="B30" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C30" s="6" t="n">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>1343</v>
+      </c>
+      <c r="C30" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D30" s="6" t="inlineStr">
+      <c r="D30" s="7" t="inlineStr">
         <is>
           <t>Price at Proven Support Zone</t>
         </is>
       </c>
-      <c r="E30" s="7" t="inlineStr">
+      <c r="E30" s="8" t="inlineStr">
         <is>
           <t>NOT MET</t>
         </is>
       </c>
-      <c r="F30" s="6" t="inlineStr">
+      <c r="F30" s="7" t="inlineStr">
         <is>
           <t>Nearest support: ₹1308.67</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>LT</t>
-        </is>
-      </c>
-      <c r="B31" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C31" s="6" t="n">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>1343</v>
+      </c>
+      <c r="C31" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D31" s="6" t="inlineStr">
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t>Bullish Reversal Candle at Support</t>
         </is>
       </c>
-      <c r="E31" s="7" t="inlineStr">
+      <c r="E31" s="8" t="inlineStr">
         <is>
           <t>NOT MET</t>
         </is>
       </c>
-      <c r="F31" s="6" t="inlineStr">
+      <c r="F31" s="7" t="inlineStr">
         <is>
           <t>BEARISH_CANDLE – Solid red candle – sellers in control.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>LT</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C32" s="6" t="n">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="n">
+        <v>1343</v>
+      </c>
+      <c r="C32" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D32" s="6" t="inlineStr">
+      <c r="D32" s="7" t="inlineStr">
         <is>
           <t>Support Zone Reaction Count ≥ 2</t>
         </is>
       </c>
-      <c r="E32" s="8" t="inlineStr">
+      <c r="E32" s="9" t="inlineStr">
         <is>
           <t>MET</t>
         </is>
       </c>
-      <c r="F32" s="6" t="inlineStr">
+      <c r="F32" s="7" t="inlineStr">
         <is>
           <t>Touch count: 7 (Major Zone)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="inlineStr">
-        <is>
-          <t>LT</t>
-        </is>
-      </c>
-      <c r="B33" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C33" s="6" t="n">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="n">
+        <v>1343</v>
+      </c>
+      <c r="C33" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D33" s="6" t="inlineStr">
+      <c r="D33" s="7" t="inlineStr">
         <is>
           <t>RR Ratio ≥ 1.5 to First Target</t>
         </is>
       </c>
-      <c r="E33" s="7" t="inlineStr">
+      <c r="E33" s="8" t="inlineStr">
         <is>
           <t>NOT MET</t>
         </is>
       </c>
-      <c r="F33" s="6" t="inlineStr">
-        <is>
-          <t>RR T1: 0.45 (POOR)</t>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>RR T1: 0.46 (POOR)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t>LT</t>
-        </is>
-      </c>
-      <c r="B34" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C34" s="6" t="n">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="n">
+        <v>1343</v>
+      </c>
+      <c r="C34" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D34" s="6" t="inlineStr">
+      <c r="D34" s="7" t="inlineStr">
         <is>
           <t>Clear Path to T1 (No Major Resistance)</t>
         </is>
       </c>
-      <c r="E34" s="7" t="inlineStr">
+      <c r="E34" s="8" t="inlineStr">
         <is>
           <t>NOT MET</t>
         </is>
       </c>
-      <c r="F34" s="6" t="inlineStr">
+      <c r="F34" s="7" t="inlineStr">
         <is>
           <t>T1 resistance: ₹1362.82</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t>LT</t>
-        </is>
-      </c>
-      <c r="B35" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C35" s="6" t="n">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="n">
+        <v>1343</v>
+      </c>
+      <c r="C35" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D35" s="6" t="inlineStr">
+      <c r="D35" s="7" t="inlineStr">
         <is>
           <t>Consolidation / Breakout Structure</t>
         </is>
       </c>
-      <c r="E35" s="8" t="inlineStr">
+      <c r="E35" s="9" t="inlineStr">
         <is>
           <t>MET</t>
         </is>
       </c>
-      <c r="F35" s="6" t="inlineStr">
+      <c r="F35" s="7" t="inlineStr">
         <is>
           <t>Inside bar or low-volatility compression visible.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>LT</t>
-        </is>
-      </c>
-      <c r="B36" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C36" s="6" t="n">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>ICICIBANK</t>
+        </is>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>1343</v>
+      </c>
+      <c r="C36" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="D36" s="6" t="inlineStr">
+      <c r="D36" s="7" t="inlineStr">
         <is>
           <t>Volume Expansion on Signal Candle</t>
         </is>
       </c>
-      <c r="E36" s="7" t="inlineStr">
+      <c r="E36" s="8" t="inlineStr">
         <is>
           <t>NOT MET</t>
         </is>
       </c>
-      <c r="F36" s="6" t="inlineStr">
-        <is>
-          <t>Last vol: 3,381,205 vs 20-day avg: 18,507,370</t>
-        </is>
-      </c>
-    </row>
-    <row r="37"/>
-    <row r="38">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>ASIANPAINT</t>
-        </is>
-      </c>
-      <c r="B38" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C38" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D38" s="6" t="inlineStr">
-        <is>
-          <t>Uptrend Confirmed (HH + HL on Daily)</t>
-        </is>
-      </c>
-      <c r="E38" s="7" t="inlineStr">
-        <is>
-          <t>NOT MET</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="inlineStr">
-        <is>
-          <t>Mixed swing points – no clear trend bias.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t>ASIANPAINT</t>
-        </is>
-      </c>
-      <c r="B39" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C39" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D39" s="6" t="inlineStr">
-        <is>
-          <t>Price at Proven Support Zone</t>
-        </is>
-      </c>
-      <c r="E39" s="7" t="inlineStr">
-        <is>
-          <t>NOT MET</t>
-        </is>
-      </c>
-      <c r="F39" s="6" t="inlineStr">
-        <is>
-          <t>Nearest support: ₹1308.67</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t>ASIANPAINT</t>
-        </is>
-      </c>
-      <c r="B40" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C40" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D40" s="6" t="inlineStr">
-        <is>
-          <t>Bullish Reversal Candle at Support</t>
-        </is>
-      </c>
-      <c r="E40" s="7" t="inlineStr">
-        <is>
-          <t>NOT MET</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="inlineStr">
-        <is>
-          <t>BEARISH_CANDLE – Solid red candle – sellers in control.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>ASIANPAINT</t>
-        </is>
-      </c>
-      <c r="B41" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C41" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D41" s="6" t="inlineStr">
-        <is>
-          <t>Support Zone Reaction Count ≥ 2</t>
-        </is>
-      </c>
-      <c r="E41" s="8" t="inlineStr">
-        <is>
-          <t>MET</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="inlineStr">
-        <is>
-          <t>Touch count: 7 (Major Zone)</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="6" t="inlineStr">
-        <is>
-          <t>ASIANPAINT</t>
-        </is>
-      </c>
-      <c r="B42" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C42" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D42" s="6" t="inlineStr">
-        <is>
-          <t>RR Ratio ≥ 1.5 to First Target</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="inlineStr">
-        <is>
-          <t>NOT MET</t>
-        </is>
-      </c>
-      <c r="F42" s="6" t="inlineStr">
-        <is>
-          <t>RR T1: 0.45 (POOR)</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t>ASIANPAINT</t>
-        </is>
-      </c>
-      <c r="B43" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C43" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D43" s="6" t="inlineStr">
-        <is>
-          <t>Clear Path to T1 (No Major Resistance)</t>
-        </is>
-      </c>
-      <c r="E43" s="7" t="inlineStr">
-        <is>
-          <t>NOT MET</t>
-        </is>
-      </c>
-      <c r="F43" s="6" t="inlineStr">
-        <is>
-          <t>T1 resistance: ₹1362.82</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="6" t="inlineStr">
-        <is>
-          <t>ASIANPAINT</t>
-        </is>
-      </c>
-      <c r="B44" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C44" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D44" s="6" t="inlineStr">
-        <is>
-          <t>Consolidation / Breakout Structure</t>
-        </is>
-      </c>
-      <c r="E44" s="8" t="inlineStr">
-        <is>
-          <t>MET</t>
-        </is>
-      </c>
-      <c r="F44" s="6" t="inlineStr">
-        <is>
-          <t>Inside bar or low-volatility compression visible.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="6" t="inlineStr">
-        <is>
-          <t>ASIANPAINT</t>
-        </is>
-      </c>
-      <c r="B45" s="6" t="n">
-        <v>1343.4</v>
-      </c>
-      <c r="C45" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D45" s="6" t="inlineStr">
-        <is>
-          <t>Volume Expansion on Signal Candle</t>
-        </is>
-      </c>
-      <c r="E45" s="7" t="inlineStr">
-        <is>
-          <t>NOT MET</t>
-        </is>
-      </c>
-      <c r="F45" s="6" t="inlineStr">
-        <is>
-          <t>Last vol: 3,381,205 vs 20-day avg: 18,507,370</t>
+      <c r="F36" s="7" t="inlineStr">
+        <is>
+          <t>Last vol: 3,575,784 vs 20-day avg: 18,517,099</t>
         </is>
       </c>
     </row>
@@ -2654,7 +2350,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Institutional Swing Analyzer – Run Metadata</t>
         </is>
@@ -2662,120 +2358,120 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Report Generated</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
-        <is>
-          <t>15-May-2026 09:43:15</t>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>15-May-2026 09:49:24</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>Analysis Framework</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>Institutional Swing Analyzer v2.0</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>Universe</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>NSE Equities (India)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>Timeframe</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Daily (1D)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>Lookback Period</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>6 Months</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>Stocks Scanned</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>5</t>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Processing Time (s)</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>0.7</t>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>1.0</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Capital Assumed</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>₹500,000</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Risk Per Trade</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>1.0%</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>SEBI Disclaimer</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>This report is for educational purposes only. Data may have a 30-day lag for unregistered entities. Not investment advice. Consult a SEBI-registered advisor.</t>
         </is>

</xml_diff>